<commit_message>
update on guide & home page nav banner
Updated the guide section (quality check & corrections) & minor updates across main pages (removed location line & nav bar update)
</commit_message>
<xml_diff>
--- a/guide/templates-tools/climate-health-materiality-tracker.xlsx
+++ b/guide/templates-tools/climate-health-materiality-tracker.xlsx
@@ -301,68 +301,72 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -621,115 +625,115 @@
   <dimension ref="B2:H21"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="3"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="100"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="3"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="100"/>
   </cols>
   <sheetData>
     <row r="2" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="2" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="3" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="4" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="C6" s="4"/>
-      <c r="D6" s="4"/>
-      <c r="E6" s="4"/>
-      <c r="F6" s="4"/>
-      <c r="G6" s="4"/>
-      <c r="H6" s="4"/>
+      <c r="C6" s="5"/>
+      <c r="D6" s="5"/>
+      <c r="E6" s="5"/>
+      <c r="F6" s="5"/>
+      <c r="G6" s="5"/>
+      <c r="H6" s="5"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B8" s="3" t="s">
+      <c r="B8" s="4" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C9" s="4"/>
-      <c r="D9" s="4"/>
-      <c r="E9" s="4"/>
-      <c r="F9" s="4"/>
-      <c r="G9" s="4"/>
-      <c r="H9" s="4"/>
+      <c r="C9" s="5"/>
+      <c r="D9" s="5"/>
+      <c r="E9" s="5"/>
+      <c r="F9" s="5"/>
+      <c r="G9" s="5"/>
+      <c r="H9" s="5"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="3" t="s">
+      <c r="B11" s="4" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B12" s="4" t="s">
+      <c r="B12" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C12" s="4"/>
-      <c r="D12" s="4"/>
-      <c r="E12" s="4"/>
-      <c r="F12" s="4"/>
-      <c r="G12" s="4"/>
-      <c r="H12" s="4"/>
+      <c r="C12" s="5"/>
+      <c r="D12" s="5"/>
+      <c r="E12" s="5"/>
+      <c r="F12" s="5"/>
+      <c r="G12" s="5"/>
+      <c r="H12" s="5"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="3" t="s">
+      <c r="B14" s="4" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B15" s="4" t="s">
+      <c r="B15" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="C15" s="4"/>
-      <c r="D15" s="4"/>
-      <c r="E15" s="4"/>
-      <c r="F15" s="4"/>
-      <c r="G15" s="4"/>
-      <c r="H15" s="4"/>
+      <c r="C15" s="5"/>
+      <c r="D15" s="5"/>
+      <c r="E15" s="5"/>
+      <c r="F15" s="5"/>
+      <c r="G15" s="5"/>
+      <c r="H15" s="5"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="3" t="s">
+      <c r="B17" s="4" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B18" s="4" t="s">
+      <c r="B18" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="C18" s="4"/>
-      <c r="D18" s="4"/>
-      <c r="E18" s="4"/>
-      <c r="F18" s="4"/>
-      <c r="G18" s="4"/>
-      <c r="H18" s="4"/>
+      <c r="C18" s="5"/>
+      <c r="D18" s="5"/>
+      <c r="E18" s="5"/>
+      <c r="F18" s="5"/>
+      <c r="G18" s="5"/>
+      <c r="H18" s="5"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B20" s="3" t="s">
+      <c r="B20" s="4" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B21" s="4" t="s">
+      <c r="B21" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="C21" s="4"/>
-      <c r="D21" s="4"/>
-      <c r="E21" s="4"/>
-      <c r="F21" s="4"/>
-      <c r="G21" s="4"/>
-      <c r="H21" s="4"/>
+      <c r="C21" s="5"/>
+      <c r="D21" s="5"/>
+      <c r="E21" s="5"/>
+      <c r="F21" s="5"/>
+      <c r="G21" s="5"/>
+      <c r="H21" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -758,412 +762,412 @@
   <dimension ref="A2:G30"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="48"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="40"/>
   </cols>
   <sheetData>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="C2" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="D2" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="E2" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="F2" s="5" t="s">
+      <c r="F2" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="G2" s="5" t="s">
+      <c r="G2" s="6" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="6" t="s">
+      <c r="A3" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="C3" s="7" t="n">
+      <c r="C3" s="8" t="n">
         <v>4</v>
       </c>
-      <c r="D3" s="7" t="n">
+      <c r="D3" s="8" t="n">
         <v>4</v>
       </c>
-      <c r="E3" s="8" t="n">
+      <c r="E3" s="9" t="n">
         <f aca="false">C3*D3</f>
         <v>16</v>
       </c>
-      <c r="F3" s="8" t="str">
+      <c r="F3" s="9" t="str">
         <f aca="false">IF(E3="","",IF(E3&gt;=15,"High",IF(E3&gt;=7,"Medium","Low")))</f>
         <v>High</v>
       </c>
-      <c r="G3" s="7"/>
+      <c r="G3" s="8"/>
     </row>
     <row r="4" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="6" t="s">
+      <c r="A4" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="C4" s="7" t="n">
+      <c r="C4" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="D4" s="7" t="n">
+      <c r="D4" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="E4" s="8" t="n">
+      <c r="E4" s="9" t="n">
         <f aca="false">C4*D4</f>
         <v>15</v>
       </c>
-      <c r="F4" s="8" t="str">
+      <c r="F4" s="9" t="str">
         <f aca="false">IF(E4="","",IF(E4&gt;=15,"High",IF(E4&gt;=7,"Medium","Low")))</f>
         <v>High</v>
       </c>
-      <c r="G4" s="7"/>
+      <c r="G4" s="8"/>
     </row>
     <row r="5" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="6" t="s">
+      <c r="A5" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="C5" s="7" t="n">
+      <c r="C5" s="8" t="n">
         <v>4</v>
       </c>
-      <c r="D5" s="7" t="n">
+      <c r="D5" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="E5" s="8" t="n">
+      <c r="E5" s="9" t="n">
         <f aca="false">C5*D5</f>
         <v>12</v>
       </c>
-      <c r="F5" s="8" t="str">
+      <c r="F5" s="9" t="str">
         <f aca="false">IF(E5="","",IF(E5&gt;=15,"High",IF(E5&gt;=7,"Medium","Low")))</f>
         <v>Medium</v>
       </c>
-      <c r="G5" s="7"/>
+      <c r="G5" s="8"/>
     </row>
     <row r="6" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="6" t="s">
+      <c r="A6" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="C6" s="7" t="n">
+      <c r="C6" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="D6" s="7" t="n">
+      <c r="D6" s="8" t="n">
         <v>4</v>
       </c>
-      <c r="E6" s="8" t="n">
+      <c r="E6" s="9" t="n">
         <f aca="false">C6*D6</f>
         <v>12</v>
       </c>
-      <c r="F6" s="8" t="str">
+      <c r="F6" s="9" t="str">
         <f aca="false">IF(E6="","",IF(E6&gt;=15,"High",IF(E6&gt;=7,"Medium","Low")))</f>
         <v>Medium</v>
       </c>
-      <c r="G6" s="7"/>
+      <c r="G6" s="8"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="9"/>
-      <c r="B7" s="9"/>
-      <c r="C7" s="10"/>
-      <c r="D7" s="10"/>
-      <c r="E7" s="11" t="str">
+      <c r="A7" s="10"/>
+      <c r="B7" s="10"/>
+      <c r="C7" s="11"/>
+      <c r="D7" s="11"/>
+      <c r="E7" s="12" t="str">
         <f aca="false">IF(OR(C7="",D7=""),"",C7*D7)</f>
         <v/>
       </c>
-      <c r="F7" s="11" t="str">
+      <c r="F7" s="12" t="str">
         <f aca="false">IF(E7="","",IF(E7&gt;=15,"High",IF(E7&gt;=7,"Medium","Low")))</f>
         <v/>
       </c>
-      <c r="G7" s="10"/>
+      <c r="G7" s="11"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="9"/>
-      <c r="B8" s="9"/>
-      <c r="C8" s="10"/>
-      <c r="D8" s="10"/>
-      <c r="E8" s="11" t="str">
+      <c r="A8" s="10"/>
+      <c r="B8" s="10"/>
+      <c r="C8" s="11"/>
+      <c r="D8" s="11"/>
+      <c r="E8" s="12" t="str">
         <f aca="false">IF(OR(C8="",D8=""),"",C8*D8)</f>
         <v/>
       </c>
-      <c r="F8" s="11" t="str">
+      <c r="F8" s="12" t="str">
         <f aca="false">IF(E8="","",IF(E8&gt;=15,"High",IF(E8&gt;=7,"Medium","Low")))</f>
         <v/>
       </c>
-      <c r="G8" s="10"/>
+      <c r="G8" s="11"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="9"/>
-      <c r="B9" s="9"/>
-      <c r="C9" s="10"/>
-      <c r="D9" s="10"/>
-      <c r="E9" s="11" t="str">
+      <c r="A9" s="10"/>
+      <c r="B9" s="10"/>
+      <c r="C9" s="11"/>
+      <c r="D9" s="11"/>
+      <c r="E9" s="12" t="str">
         <f aca="false">IF(OR(C9="",D9=""),"",C9*D9)</f>
         <v/>
       </c>
-      <c r="F9" s="11" t="str">
+      <c r="F9" s="12" t="str">
         <f aca="false">IF(E9="","",IF(E9&gt;=15,"High",IF(E9&gt;=7,"Medium","Low")))</f>
         <v/>
       </c>
-      <c r="G9" s="10"/>
+      <c r="G9" s="11"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="9"/>
-      <c r="B10" s="9"/>
-      <c r="C10" s="10"/>
-      <c r="D10" s="10"/>
-      <c r="E10" s="11" t="str">
+      <c r="A10" s="10"/>
+      <c r="B10" s="10"/>
+      <c r="C10" s="11"/>
+      <c r="D10" s="11"/>
+      <c r="E10" s="12" t="str">
         <f aca="false">IF(OR(C10="",D10=""),"",C10*D10)</f>
         <v/>
       </c>
-      <c r="F10" s="11" t="str">
+      <c r="F10" s="12" t="str">
         <f aca="false">IF(E10="","",IF(E10&gt;=15,"High",IF(E10&gt;=7,"Medium","Low")))</f>
         <v/>
       </c>
-      <c r="G10" s="10"/>
+      <c r="G10" s="11"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="9"/>
-      <c r="B11" s="9"/>
-      <c r="C11" s="10"/>
-      <c r="D11" s="10"/>
-      <c r="E11" s="11" t="str">
+      <c r="A11" s="10"/>
+      <c r="B11" s="10"/>
+      <c r="C11" s="11"/>
+      <c r="D11" s="11"/>
+      <c r="E11" s="12" t="str">
         <f aca="false">IF(OR(C11="",D11=""),"",C11*D11)</f>
         <v/>
       </c>
-      <c r="F11" s="11" t="str">
+      <c r="F11" s="12" t="str">
         <f aca="false">IF(E11="","",IF(E11&gt;=15,"High",IF(E11&gt;=7,"Medium","Low")))</f>
         <v/>
       </c>
-      <c r="G11" s="10"/>
+      <c r="G11" s="11"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="9"/>
-      <c r="B12" s="9"/>
-      <c r="C12" s="10"/>
-      <c r="D12" s="10"/>
-      <c r="E12" s="11" t="str">
+      <c r="A12" s="10"/>
+      <c r="B12" s="10"/>
+      <c r="C12" s="11"/>
+      <c r="D12" s="11"/>
+      <c r="E12" s="12" t="str">
         <f aca="false">IF(OR(C12="",D12=""),"",C12*D12)</f>
         <v/>
       </c>
-      <c r="F12" s="11" t="str">
+      <c r="F12" s="12" t="str">
         <f aca="false">IF(E12="","",IF(E12&gt;=15,"High",IF(E12&gt;=7,"Medium","Low")))</f>
         <v/>
       </c>
-      <c r="G12" s="10"/>
+      <c r="G12" s="11"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="9"/>
-      <c r="B13" s="9"/>
-      <c r="C13" s="10"/>
-      <c r="D13" s="10"/>
-      <c r="E13" s="11" t="str">
+      <c r="A13" s="10"/>
+      <c r="B13" s="10"/>
+      <c r="C13" s="11"/>
+      <c r="D13" s="11"/>
+      <c r="E13" s="12" t="str">
         <f aca="false">IF(OR(C13="",D13=""),"",C13*D13)</f>
         <v/>
       </c>
-      <c r="F13" s="11" t="str">
+      <c r="F13" s="12" t="str">
         <f aca="false">IF(E13="","",IF(E13&gt;=15,"High",IF(E13&gt;=7,"Medium","Low")))</f>
         <v/>
       </c>
-      <c r="G13" s="10"/>
+      <c r="G13" s="11"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="9"/>
-      <c r="B14" s="9"/>
-      <c r="C14" s="10"/>
-      <c r="D14" s="10"/>
-      <c r="E14" s="11" t="str">
+      <c r="A14" s="10"/>
+      <c r="B14" s="10"/>
+      <c r="C14" s="11"/>
+      <c r="D14" s="11"/>
+      <c r="E14" s="12" t="str">
         <f aca="false">IF(OR(C14="",D14=""),"",C14*D14)</f>
         <v/>
       </c>
-      <c r="F14" s="11" t="str">
+      <c r="F14" s="12" t="str">
         <f aca="false">IF(E14="","",IF(E14&gt;=15,"High",IF(E14&gt;=7,"Medium","Low")))</f>
         <v/>
       </c>
-      <c r="G14" s="10"/>
+      <c r="G14" s="11"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="9"/>
-      <c r="B15" s="9"/>
-      <c r="C15" s="10"/>
-      <c r="D15" s="10"/>
-      <c r="E15" s="11" t="str">
+      <c r="A15" s="10"/>
+      <c r="B15" s="10"/>
+      <c r="C15" s="11"/>
+      <c r="D15" s="11"/>
+      <c r="E15" s="12" t="str">
         <f aca="false">IF(OR(C15="",D15=""),"",C15*D15)</f>
         <v/>
       </c>
-      <c r="F15" s="11" t="str">
+      <c r="F15" s="12" t="str">
         <f aca="false">IF(E15="","",IF(E15&gt;=15,"High",IF(E15&gt;=7,"Medium","Low")))</f>
         <v/>
       </c>
-      <c r="G15" s="10"/>
+      <c r="G15" s="11"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="9"/>
-      <c r="B16" s="9"/>
-      <c r="C16" s="10"/>
-      <c r="D16" s="10"/>
-      <c r="E16" s="11" t="str">
+      <c r="A16" s="10"/>
+      <c r="B16" s="10"/>
+      <c r="C16" s="11"/>
+      <c r="D16" s="11"/>
+      <c r="E16" s="12" t="str">
         <f aca="false">IF(OR(C16="",D16=""),"",C16*D16)</f>
         <v/>
       </c>
-      <c r="F16" s="11" t="str">
+      <c r="F16" s="12" t="str">
         <f aca="false">IF(E16="","",IF(E16&gt;=15,"High",IF(E16&gt;=7,"Medium","Low")))</f>
         <v/>
       </c>
-      <c r="G16" s="10"/>
+      <c r="G16" s="11"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="9"/>
-      <c r="B17" s="9"/>
-      <c r="C17" s="10"/>
-      <c r="D17" s="10"/>
-      <c r="E17" s="11" t="str">
+      <c r="A17" s="10"/>
+      <c r="B17" s="10"/>
+      <c r="C17" s="11"/>
+      <c r="D17" s="11"/>
+      <c r="E17" s="12" t="str">
         <f aca="false">IF(OR(C17="",D17=""),"",C17*D17)</f>
         <v/>
       </c>
-      <c r="F17" s="11" t="str">
+      <c r="F17" s="12" t="str">
         <f aca="false">IF(E17="","",IF(E17&gt;=15,"High",IF(E17&gt;=7,"Medium","Low")))</f>
         <v/>
       </c>
-      <c r="G17" s="10"/>
+      <c r="G17" s="11"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="9"/>
-      <c r="B18" s="9"/>
-      <c r="C18" s="10"/>
-      <c r="D18" s="10"/>
-      <c r="E18" s="11" t="str">
+      <c r="A18" s="10"/>
+      <c r="B18" s="10"/>
+      <c r="C18" s="11"/>
+      <c r="D18" s="11"/>
+      <c r="E18" s="12" t="str">
         <f aca="false">IF(OR(C18="",D18=""),"",C18*D18)</f>
         <v/>
       </c>
-      <c r="F18" s="11" t="str">
+      <c r="F18" s="12" t="str">
         <f aca="false">IF(E18="","",IF(E18&gt;=15,"High",IF(E18&gt;=7,"Medium","Low")))</f>
         <v/>
       </c>
-      <c r="G18" s="10"/>
+      <c r="G18" s="11"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="9"/>
-      <c r="B19" s="9"/>
-      <c r="C19" s="10"/>
-      <c r="D19" s="10"/>
-      <c r="E19" s="11" t="str">
+      <c r="A19" s="10"/>
+      <c r="B19" s="10"/>
+      <c r="C19" s="11"/>
+      <c r="D19" s="11"/>
+      <c r="E19" s="12" t="str">
         <f aca="false">IF(OR(C19="",D19=""),"",C19*D19)</f>
         <v/>
       </c>
-      <c r="F19" s="11" t="str">
+      <c r="F19" s="12" t="str">
         <f aca="false">IF(E19="","",IF(E19&gt;=15,"High",IF(E19&gt;=7,"Medium","Low")))</f>
         <v/>
       </c>
-      <c r="G19" s="10"/>
+      <c r="G19" s="11"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="9"/>
-      <c r="B20" s="9"/>
-      <c r="C20" s="10"/>
-      <c r="D20" s="10"/>
-      <c r="E20" s="11" t="str">
+      <c r="A20" s="10"/>
+      <c r="B20" s="10"/>
+      <c r="C20" s="11"/>
+      <c r="D20" s="11"/>
+      <c r="E20" s="12" t="str">
         <f aca="false">IF(OR(C20="",D20=""),"",C20*D20)</f>
         <v/>
       </c>
-      <c r="F20" s="11" t="str">
+      <c r="F20" s="12" t="str">
         <f aca="false">IF(E20="","",IF(E20&gt;=15,"High",IF(E20&gt;=7,"Medium","Low")))</f>
         <v/>
       </c>
-      <c r="G20" s="10"/>
+      <c r="G20" s="11"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="9"/>
-      <c r="B21" s="9"/>
-      <c r="C21" s="10"/>
-      <c r="D21" s="10"/>
-      <c r="E21" s="11" t="str">
+      <c r="A21" s="10"/>
+      <c r="B21" s="10"/>
+      <c r="C21" s="11"/>
+      <c r="D21" s="11"/>
+      <c r="E21" s="12" t="str">
         <f aca="false">IF(OR(C21="",D21=""),"",C21*D21)</f>
         <v/>
       </c>
-      <c r="F21" s="11" t="str">
+      <c r="F21" s="12" t="str">
         <f aca="false">IF(E21="","",IF(E21&gt;=15,"High",IF(E21&gt;=7,"Medium","Low")))</f>
         <v/>
       </c>
-      <c r="G21" s="10"/>
+      <c r="G21" s="11"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="9"/>
-      <c r="B22" s="9"/>
-      <c r="C22" s="10"/>
-      <c r="D22" s="10"/>
-      <c r="E22" s="11" t="str">
+      <c r="A22" s="10"/>
+      <c r="B22" s="10"/>
+      <c r="C22" s="11"/>
+      <c r="D22" s="11"/>
+      <c r="E22" s="12" t="str">
         <f aca="false">IF(OR(C22="",D22=""),"",C22*D22)</f>
         <v/>
       </c>
-      <c r="F22" s="11" t="str">
+      <c r="F22" s="12" t="str">
         <f aca="false">IF(E22="","",IF(E22&gt;=15,"High",IF(E22&gt;=7,"Medium","Low")))</f>
         <v/>
       </c>
-      <c r="G22" s="10"/>
+      <c r="G22" s="11"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="12" t="s">
+      <c r="A25" s="13" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="13" t="s">
+      <c r="A26" s="14" t="s">
         <v>30</v>
       </c>
-      <c r="B26" s="14" t="n">
+      <c r="B26" s="15" t="n">
         <f aca="false">COUNTIF(F3:F22,"High")</f>
         <v>2</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="13" t="s">
+      <c r="A27" s="14" t="s">
         <v>31</v>
       </c>
-      <c r="B27" s="14" t="n">
+      <c r="B27" s="15" t="n">
         <f aca="false">COUNTIF(F3:F22,"Medium")</f>
         <v>2</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="13" t="s">
+      <c r="A28" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="B28" s="14" t="n">
+      <c r="B28" s="15" t="n">
         <f aca="false">COUNTIF(F3:F22,"Low")</f>
         <v>0</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="15" t="s">
+      <c r="A30" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="B30" s="15"/>
-      <c r="C30" s="15"/>
-      <c r="D30" s="15"/>
-      <c r="E30" s="15"/>
-      <c r="F30" s="15"/>
-      <c r="G30" s="15"/>
+      <c r="B30" s="16"/>
+      <c r="C30" s="16"/>
+      <c r="D30" s="16"/>
+      <c r="E30" s="16"/>
+      <c r="F30" s="16"/>
+      <c r="G30" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>